<commit_message>
Update Tennis PostPlanner XLSX with regenerated timestamps for 2026-07-27
Regenerated during Parenting pipeline run to verify script compatibility; post times shifted from 12:57–20:39 to 13:13–20:43 ET (same 7 posts, same content).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MJn5fZ8MJcrvxTpS8jkkMx
</commit_message>
<xml_diff>
--- a/Tennis/postplanner-imports/tfr-postplanner-2026-07-27.xlsx
+++ b/Tennis/postplanner-imports/tfr-postplanner-2026-07-27.xlsx
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>07/27/2026  12:57</t>
+          <t>07/27/2026  13:13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -494,7 +494,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>07/27/2026  14:14</t>
+          <t>07/27/2026  14:28</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -512,7 +512,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>07/27/2026  15:31</t>
+          <t>07/27/2026  15:43</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -528,7 +528,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>07/27/2026  16:48</t>
+          <t>07/27/2026  16:58</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -544,7 +544,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>07/27/2026  18:05</t>
+          <t>07/27/2026  18:13</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -560,7 +560,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07/27/2026  19:22</t>
+          <t>07/27/2026  19:28</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -576,7 +576,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07/27/2026  20:39</t>
+          <t>07/27/2026  20:43</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">

</xml_diff>